<commit_message>
Saving progress with mission construction
</commit_message>
<xml_diff>
--- a/SizingCodeV2/Lookups/engine_lookup.xlsx
+++ b/SizingCodeV2/Lookups/engine_lookup.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfile\Documents\MyDocuments\CODING\GitWorkingDirectory\team10aiaa\Sizing Code V2\Lookups\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfile\Documents\MyDocuments\CODING\GitWorkingDirectory\team10aiaa\SizingCodeV2\Lookups\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35E24E00-933E-43B5-90B4-9F6446BD0AB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97404404-1BB8-4FCB-B95B-F64C210BB4F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -122,10 +122,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -461,6 +462,7 @@
       <c r="C2">
         <v>78700</v>
       </c>
+      <c r="D2" s="3"/>
       <c r="E2">
         <v>26</v>
       </c>
@@ -494,6 +496,7 @@
       <c r="C3">
         <v>191000</v>
       </c>
+      <c r="D3" s="3"/>
       <c r="E3">
         <v>28</v>
       </c>
@@ -526,7 +529,7 @@
       <c r="C4">
         <v>92207.185546399996</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="3">
         <v>4.8600000000000003</v>
       </c>
       <c r="E4">
@@ -561,7 +564,7 @@
       <c r="C5">
         <v>129600</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="3">
         <f>6948900/1000000</f>
         <v>6.9489000000000001</v>
       </c>
@@ -598,6 +601,10 @@
       <c r="C6">
         <v>144600</v>
       </c>
+      <c r="D6" s="3">
+        <f>4.86*1.2</f>
+        <v>5.8319999999999999</v>
+      </c>
       <c r="E6">
         <v>30.4</v>
       </c>
@@ -631,6 +638,7 @@
       <c r="C7">
         <v>480</v>
       </c>
+      <c r="D7" s="3"/>
       <c r="E7">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
In the middle of tuning settings
</commit_message>
<xml_diff>
--- a/SizingCodeV2/Lookups/engine_lookup.xlsx
+++ b/SizingCodeV2/Lookups/engine_lookup.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfile\Documents\MyDocuments\CODING\GitWorkingDirectory\team10aiaa\SizingCodeV2\Lookups\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97404404-1BB8-4FCB-B95B-F64C210BB4F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1510716-9B22-4797-B579-0717BD4009A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>F404</t>
   </si>
@@ -87,6 +87,9 @@
   </si>
   <si>
     <t>Cost_mil</t>
+  </si>
+  <si>
+    <t>TF41-A-2</t>
   </si>
 </sst>
 </file>
@@ -407,7 +410,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.5546875" customWidth="1"/>
@@ -662,6 +665,26 @@
         <v>0.111</v>
       </c>
     </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8">
+        <v>66723</v>
+      </c>
+      <c r="C8">
+        <v>66800</v>
+      </c>
+      <c r="D8">
+        <v>3</v>
+      </c>
+      <c r="J8">
+        <v>15618</v>
+      </c>
+      <c r="K8">
+        <v>0.94440000000000002</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>